<commit_message>
Merge concurrent research checkpoints without data loss
</commit_message>
<xml_diff>
--- a/output/review.xlsx
+++ b/output/review.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE1"/>
+  <dimension ref="A1:AF1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -559,17 +559,22 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
+          <t>merged_checkpoint_rows</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>identity_url</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>previous_status</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
           <t>physician_search_version</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>identity_url</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>previous_status</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recover contacts and guard verified history
</commit_message>
<xml_diff>
--- a/output/review.xlsx
+++ b/output/review.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,178 +413,198 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH1"/>
+  <dimension ref="A1:AL1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>algo_version</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>physician_search_version</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>priority</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>target_kind</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>seed_source</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>license_number</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>seed_type</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>email_type</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>source_url</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>evidence</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>matched_query</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>extraction_method</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>alternate_emails</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>candidate_count</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>retry_count</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>next_retry_at</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>last_attempt_at</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>search_queries</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>search_errors</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>search_results</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>pages_fetched</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>fetch_failures</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>search_provider</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>attempted_urls</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>merged_checkpoint_rows</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>shared_target_count</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>unchanged_search_count</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
         <is>
           <t>identity_url</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>previous_status</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>verification_review_required</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>previous_candidate</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>resolution_reason</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>search_fingerprint</t>
         </is>
       </c>
     </row>

</xml_diff>